<commit_message>
Code review + changes
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cristi/Desktop/Facultate/Anul_III_Sem_II/VVSS/Lab VVSS - Echipa AM16/docs/Lab01/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2026_1\UBB\VVSS\Laboratoare\GitLab\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1616022D-6E37-7A41-B43F-8339300EA557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="32180" windowHeight="19520" tabRatio="650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="32183" windowHeight="19523" tabRatio="650" firstSheet="1" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -18,25 +17,12 @@
     <sheet name="Coding Phase Defects" sheetId="5" r:id="rId3"/>
     <sheet name="Tool-basedCodeAnalysis" sheetId="8" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="104">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -319,13 +305,170 @@
   </si>
   <si>
     <t>.toList();</t>
+  </si>
+  <si>
+    <t>C01</t>
+  </si>
+  <si>
+    <t>ProductService</t>
+  </si>
+  <si>
+    <t>În metodele de adăugare a produselor sau ingredientelor, lipsește validarea valorilor numerice. De exemplu, sistemul permite introducerea unui preț negativ sau a unui volum de 0 ml, ceea ce ar corupe logica financiară și de stoc. În ProductService, înainte de a trimite obiectul către Repository, adăugarea unei validări explicite: if (price &lt;= 0) throw new ValidationException("Prețul trebuie să fie pozitiv"); Aceeași logică se aplică și volumului.</t>
+  </si>
+  <si>
+    <t>C04</t>
+  </si>
+  <si>
+    <t>FileRepository</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">În clasele de tip </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FileRepository</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (ex: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>FileProductRepository</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">), citirea din fișier se face probabil prin </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>split(",")</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Dacă o linie din fișierul text este goală sau are un format corupt (un câmp lipsește), aplicația va genera un </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ArrayIndexOutOfBoundsException</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> și se va prăbuși la pornire. Îmbunătațire: verificare a lungimii array-ului rezultat după split.</t>
+    </r>
+  </si>
+  <si>
+    <t>OrderService</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Logica de verificare a stocului (înainte de comandă) trebuie să fie cumulativă. Dacă o comandă conține două băuturi diferite care folosesc același ingredient (ex: zahăr), sistemul trebuie să verifice dacă stocul total acoperă </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>suma</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> cantităților necesare. În OrderService, trebuie creată o metodă care să mapeze toate ingredientele necesare într-un Map&lt;Ingredient, Double&gt; (agregând cantitățile) înainte de a interoga StocService. Altfel, decizia de a procesa comanda va fi eronată dacă stocul e suficient pentru fiecare produs separat, dar nu pentru ambele împreună.</t>
+    </r>
+  </si>
+  <si>
+    <t>C07</t>
+  </si>
+  <si>
+    <t>CsvExperoter</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La generarea fișierului </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>CSV</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> pentru bonul de casă sau export, caracterele speciale din descrierea produselor (cum ar fi virgula) nu sunt gestionate. Dacă o descriere conține o virgulă, fișierul generat va avea coloanele decalate la deschiderea în Excel. În CsvExporter, toate câmpurile de tip text trebuie încadrate între ghilimele: writer.append("\"" + description + "\"");</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -408,6 +551,26 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -510,7 +673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -541,6 +704,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -583,9 +750,15 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -605,9 +778,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -645,9 +818,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -682,7 +855,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -717,7 +890,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -890,41 +1063,41 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" style="6"/>
+    <col min="1" max="1" width="8.796875" style="6"/>
     <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
     <col min="3" max="4" width="16.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.5" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.83203125" style="6"/>
+    <col min="5" max="5" width="41.46484375" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.796875" style="6"/>
     <col min="9" max="9" width="21" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.5" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.83203125" style="6"/>
+    <col min="10" max="10" width="14.46484375" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.796875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B2" s="24" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -933,73 +1106,73 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="27"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="27"/>
+      <c r="E5" s="29"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="22"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="37">
+      <c r="D7" s="23">
         <v>46089</v>
       </c>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1013,7 +1186,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="64" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="71.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1027,7 +1200,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="28.5">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1042,7 +1215,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="42.75">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
@@ -1057,7 +1230,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="28.5">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1072,7 +1245,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="47" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="47" customHeight="1">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1087,7 +1260,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="28.5">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1102,7 +1275,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="42.75">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1117,7 +1290,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1126,7 +1299,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1135,7 +1308,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1144,7 +1317,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1153,7 +1326,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1162,7 +1335,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1171,7 +1344,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1180,7 +1353,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1189,7 +1362,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1198,7 +1371,7 @@
       <c r="D25" s="3"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:5">
       <c r="C27" s="11" t="s">
         <v>8</v>
       </c>
@@ -1222,40 +1395,40 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" style="6"/>
+    <col min="1" max="1" width="8.796875" style="6"/>
     <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
     <col min="3" max="4" width="16.33203125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.5" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.83203125" style="6"/>
-    <col min="9" max="9" width="22.1640625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.83203125" style="6"/>
+    <col min="5" max="5" width="41.46484375" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.796875" style="6"/>
+    <col min="9" max="9" width="22.1328125" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.796875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B2" s="24" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1264,73 +1437,73 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="28"/>
+      <c r="E4" s="30"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="30"/>
+      <c r="E5" s="32"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="22"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="37">
+      <c r="D7" s="23">
         <v>46089</v>
       </c>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1344,7 +1517,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="42.75">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1358,7 +1531,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1367,7 +1540,7 @@
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
@@ -1376,7 +1549,7 @@
       <c r="D12" s="1"/>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1385,7 +1558,7 @@
       <c r="D13" s="1"/>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1394,7 +1567,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1403,7 +1576,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1412,7 +1585,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1421,7 +1594,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1430,7 +1603,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1439,7 +1612,7 @@
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1448,7 +1621,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1457,7 +1630,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1466,7 +1639,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1475,7 +1648,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1484,7 +1657,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1493,7 +1666,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:5">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1502,7 +1675,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:5">
       <c r="C28" s="11" t="s">
         <v>8</v>
       </c>
@@ -1524,41 +1697,41 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" style="6"/>
+    <col min="1" max="1" width="8.796875" style="6"/>
     <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
     <col min="3" max="3" width="16.33203125" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.5" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.83203125" style="6"/>
+    <col min="5" max="5" width="41.46484375" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.796875" style="6"/>
     <col min="9" max="9" width="26.6640625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.83203125" style="6"/>
+    <col min="10" max="16384" width="8.796875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B2" s="24" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1567,73 +1740,73 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="31"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="33"/>
+      <c r="E5" s="35"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="22"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="37">
+      <c r="D7" s="23">
         <v>46089</v>
       </c>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1647,42 +1820,66 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="149.25">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C10" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="40" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="114">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C11" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="E11" s="41" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="185.25">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C12" s="39" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>99</v>
+      </c>
+      <c r="E12" s="41" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="114">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="C13" s="39" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" s="41" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1691,7 +1888,7 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1700,7 +1897,7 @@
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1709,7 +1906,7 @@
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1718,7 +1915,7 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1727,7 +1924,7 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1736,7 +1933,7 @@
       <c r="D19" s="1"/>
       <c r="E19" s="2"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1745,7 +1942,7 @@
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1754,7 +1951,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="2"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1763,7 +1960,7 @@
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1772,7 +1969,7 @@
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1781,7 +1978,7 @@
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1790,7 +1987,7 @@
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:5">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1799,7 +1996,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:5">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1808,7 +2005,7 @@
       <c r="D27" s="2"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:5">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -1817,7 +2014,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:5">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -1826,7 +2023,7 @@
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:5">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -1835,12 +2032,14 @@
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:5">
       <c r="C32" s="11" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="12"/>
-      <c r="E32" s="1"/>
+      <c r="E32" s="1" t="s">
+        <v>54</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1857,42 +2056,42 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" style="6"/>
+    <col min="1" max="1" width="8.796875" style="6"/>
     <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="19.1640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="19.1328125" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="23.796875" style="6" customWidth="1"/>
     <col min="6" max="6" width="16.6640625" style="6" customWidth="1"/>
-    <col min="7" max="8" width="8.83203125" style="6"/>
+    <col min="7" max="8" width="8.796875" style="6"/>
     <col min="9" max="9" width="26.6640625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.83203125" style="6"/>
+    <col min="10" max="16384" width="8.796875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="15.75">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B2" s="24" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1901,63 +2100,63 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="36" t="s">
+      <c r="I3" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="36" t="s">
+      <c r="I4" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="22"/>
+      <c r="E5" s="24"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="22">
         <v>233</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="37">
+      <c r="D6" s="23">
         <v>46089</v>
       </c>
-      <c r="E6" s="22"/>
+      <c r="E6" s="24"/>
       <c r="F6" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1974,7 +2173,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="80" customHeight="1">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1991,7 +2190,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="94" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="94.05" customHeight="1">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -2009,7 +2208,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="96" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="85.5">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
@@ -2027,7 +2226,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="28.5">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -2045,7 +2244,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="96" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="85.5">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -2063,7 +2262,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="96" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="85.5">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2081,7 +2280,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="112" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="99.75">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2099,7 +2298,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="2:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:6" ht="42.75">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -2117,7 +2316,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="2:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:6" ht="85.5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -2135,7 +2334,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="2:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:6" ht="85.5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -2153,7 +2352,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:6">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2163,7 +2362,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:6">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2173,7 +2372,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:6">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2183,7 +2382,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:6">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2193,7 +2392,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:6">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2203,7 +2402,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:6">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2213,7 +2412,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:6">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2223,7 +2422,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:6">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -2233,7 +2432,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:6">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2243,7 +2442,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:6">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2253,7 +2452,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:6">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2263,17 +2462,17 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="C32" s="34" t="s">
+    <row r="32" spans="2:6">
+      <c r="C32" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
       <c r="F32" s="18" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="6:6">
       <c r="F35" s="21"/>
     </row>
   </sheetData>

</xml_diff>